<commit_message>
feat : 캐릭터 창 UI
</commit_message>
<xml_diff>
--- a/Client/Bin/Resources/Data/xlsx/DT_Texture.xlsx
+++ b/Client/Bin/Resources/Data/xlsx/DT_Texture.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitDesktop\Dx11_Naruto\Client\Bin\Resources\Data\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40331B1C-5F81-4F0F-9303-83327C2EC568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D09C806-C95E-4049-800D-49668CF45515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E1BA714A-44F4-4B9F-B605-6C062A1AF184}"/>
+    <workbookView xWindow="5895" yWindow="1815" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{E1BA714A-44F4-4B9F-B605-6C062A1AF184}"/>
   </bookViews>
   <sheets>
     <sheet name="Default" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="43">
   <si>
     <t>Id</t>
   </si>
@@ -72,9 +72,6 @@
   </si>
   <si>
     <t>COMPONENT_TYPE_TEXTURE_LOADING</t>
-  </si>
-  <si>
-    <t>../../Client/Bin/Resources/Textures/UI/Loading_Screen/Textures/T_UI_LoadingScreen_%03d_BC.png</t>
   </si>
   <si>
     <t>COMPONENT_TYPE_TEXTURE_SKILL_ICON</t>
@@ -162,6 +159,14 @@
   </si>
   <si>
     <t>COMPONENT_TYPE_TEXTURE_SKILL_GAUGE</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>../../Client/Bin/Resources/Textures/UI/TextUI/Common_Textures/Menu_Title/T_ui_Title_Logo_CharMake_BC_LOCL.png</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>../../Client/Bin/Resources/Textures/UI/Loading_Screen/Textures/T_UI_LoadingScreen_%d_BC.png</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1189,10 +1194,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
         <v>20</v>
-      </c>
-      <c r="B4" t="s">
-        <v>21</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -1203,10 +1208,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -1217,10 +1222,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -1308,7 +1313,7 @@
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -1317,7 +1322,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -1325,7 +1330,7 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -1346,7 +1351,7 @@
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42.625" customWidth="1"/>
-    <col min="2" max="2" width="78.875" customWidth="1"/>
+    <col min="2" max="2" width="88.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -1371,10 +1376,10 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" t="s">
         <v>10</v>
@@ -1399,10 +1404,10 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -1416,7 +1421,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5099ABA-1BAA-4011-9CAA-9DE70369DED4}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40.125" customWidth="1"/>
@@ -1444,142 +1449,156 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
         <v>29</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
         <v>30</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1617,10 +1636,10 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C2" s="2">
         <v>2</v>
@@ -1631,10 +1650,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" s="2">
         <v>5</v>

</xml_diff>